<commit_message>
FY 2025-26 financials: follow latest Tally TB - provisions, no partner loan
Tally now records Branding Expense and Business Promotion (Rs 2,25,000
each) against Provisions Rs 4,50,000, so the Rs 2,50,000 loan from
Samartha is removed. Capital stays Rs 2,00,000 with the contribution
still receivable from partners (b/f from FY 2024-25). Expense lines use
the Tally ledger names. Reconciliation workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PBFJrzW3fVaXJi95GNnthu
</commit_message>
<xml_diff>
--- a/outputs/Star_Fandom_FY2025-26_Tally_vs_Financials_vs_Winman.xlsx
+++ b/outputs/Star_Fandom_FY2025-26_Tally_vs_Financials_vs_Winman.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Tally TB as exported (TrialBal.xlsx)</t>
+          <t>Tally TB as exported (TrialBal.xlsx, latest)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -696,27 +696,27 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Unsecured loan from Samartha Raghava Nagabhushanam (long-term)</t>
+          <t>Provisions (Tally group) - Short-term provisions</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0</v>
+        <v>450000</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D8" s="7">
         <f>B8+C8</f>
         <v/>
       </c>
       <c r="E8" s="6" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="H8" s="7">
         <f>F8+G8</f>
@@ -980,27 +980,27 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Receivable from partners (capital) - opening 2,00,000 settled during the year</t>
+          <t>Receivable from partners (capital contribution)</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="D17" s="7">
         <f>B17+C17</f>
         <v/>
       </c>
       <c r="E17" s="6" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="H17" s="7">
         <f>F17+G17</f>
@@ -1405,14 +1405,14 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Business promotion</t>
+          <t>Branding Expense (Winman: 'Business Expenses')</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0</v>
+        <v>225000</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>225000</v>
+        <v>0</v>
       </c>
       <c r="D30" s="7">
         <f>B30+C30</f>
@@ -1439,14 +1439,14 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Business expenses</t>
+          <t>Business Promotion</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0</v>
+        <v>225000</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>225000</v>
+        <v>0</v>
       </c>
       <c r="D31" s="7">
         <f>B31+C31</f>
@@ -1592,26 +1592,47 @@
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>Partners' contribution (capital): Winman has one 'Partners' capital' field: contribution 2,00,000 less current account 13,719 = 1,86,281</t>
+          <t>Partners' contribution (capital): Not in Tally (no opening balances); Rs 2,00,000 b/f from signed FY 2024-25 accounts. Winman has one 'Partners' capital' field: 2,00,000 less loss 13,719 = 1,86,281</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Sponsorship Amount - Sale of services: Winman: move 9,23,729 from 'Sale of products/goods' to 'Sale of services'</t>
+          <t>Provisions (Tally group) - Short-term provisions: Tally: credit side of Branding Expense and Business Promotion (2,25,000 each)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Mobile Expenses (Telephone): Financials: 3,918.50 less Tally round off 0.22 = 3,918.28, shown as 3,918</t>
+          <t>Receivable from partners (capital contribution): B/f from FY 2024-25; still receivable. Winman: enter under 'Other current assets'</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Sponsorship Amount - Sale of services: Winman: move 9,23,729 from 'Sale of products/goods' to 'Sale of services'</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Mobile Expenses (Telephone): Financials: 3,918.50 less Tally round off 0.22 = 3,918.28, shown as 3,918</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Column B (Tally as exported) shows a difference of (13,719.42) on the check row only because the loss still sits in Tally's P&amp;L; it moves to the partners' current accounts when entry 2 on sheet 2 is posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Tally 'after entries' keeps paise; the financials and Winman are in whole rupees (nearest rupee). Winman as exported cut off the paise on Advances (.61) and Bank (.76) - that is the source of the earlier Rs 2 difference.</t>
         </is>
@@ -1641,7 +1662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1655,7 +1676,7 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>A. Entries to post in Tally (FY 2025-26) so the books agree with the financial statements</t>
+          <t>A. Entries still to post in Tally (FY 2025-26) - the Rs 4,50,000 expenses and provision are already in Tally</t>
         </is>
       </c>
     </row>
@@ -1735,21 +1756,21 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>During FY</t>
+          <t>31-03-2026</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Business promotion</t>
+          <t>Partners' Current Account - Pramod (20%)</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>225000</v>
+        <v>2743.88</v>
       </c>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Business expenses paid by partners on behalf of the LLP</t>
+          <t>Loss for the year Rs 13,719.42 (books, with paise) shared 20:50:15:15</t>
         </is>
       </c>
     </row>
@@ -1758,11 +1779,11 @@
       <c r="B7" s="8" t="inlineStr"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Business expenses</t>
+          <t>Partners' Current Account - Samartha (50%)</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>225000</v>
+        <v>6859.71</v>
       </c>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="5" t="inlineStr"/>
@@ -1772,180 +1793,184 @@
       <c r="B8" s="8" t="inlineStr"/>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   To Receivable from Partners (capital contribution) - settled</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Capital contribution of Rs 2,00,000 treated as paid</t>
-        </is>
-      </c>
+          <t>Partners' Current Account - Nithin (15%)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2057.91</v>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="8" t="inlineStr"/>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   To Unsecured Loan - Samartha Raghava Nagabhushanam (new ledger, long-term, no interest)</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="6" t="n">
-        <v>250000</v>
-      </c>
+          <t>Partners' Current Account - Varun (15%)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2057.92</v>
+      </c>
+      <c r="E9" s="7" t="n"/>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Keep separate from the existing 'Loan From Samarha...' ledger, which stays at Dr 4,09,311.61</t>
+          <t>Rounding paise placed here so the total is exact</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>31-03-2026</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="inlineStr"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Partners' Current Account - Pramod (20%)</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>2743.88</v>
-      </c>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Loss for the year Rs 13,719.42 (books, with paise) shared 20:50:15:15</t>
-        </is>
-      </c>
+          <t xml:space="preserve">   To Profit &amp; Loss A/c</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="6" t="n">
+        <v>13719.42</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Partners' Current Account - Samartha (50%)</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>6859.71</v>
-      </c>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="5" t="inlineStr"/>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Totals</t>
+        </is>
+      </c>
+      <c r="D11" s="19">
+        <f>SUM(D4:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="19">
+        <f>SUM(E4:E10)</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>IF(ABS(D11-E11)&lt;0.005,"Debits = Credits","NOT BALANCED")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="8" t="inlineStr"/>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Partners' Current Account - Nithin (15%)</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>2057.91</v>
-      </c>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Partners' Current Account - Varun (15%)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>2057.92</v>
-      </c>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Rounding paise placed here so the total is exact</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Note: the loss in the books is Rs 13,719.42; the financial statements show it rounded to Rs 13,719 (split 2,743.80 / 6,859.50 / 2,057.85 / 2,057.85).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="8" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   To Profit &amp; Loss A/c</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="6" t="n">
-        <v>13719.42</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>B. Corrections to make in Winman (ITR-5, A.Y. 2026-27)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>Totals</t>
-        </is>
-      </c>
-      <c r="D15" s="19">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="19">
-        <f>SUM(E4:E14)</f>
-        <v/>
-      </c>
-      <c r="F15">
-        <f>IF(ABS(D15-E15)&lt;0.005,"Debits = Credits","NOT BALANCED")</f>
-        <v/>
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Winman sheet / field</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>As exported</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>Change to</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Note: the loss in the books is Rs 13,719.42; the financial statements show it rounded to Rs 13,719 (split 2,743.80 / 6,859.50 / 2,057.85 / 2,057.85).</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Balance Sheet - Partners' / Members' capital</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>186281</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Contribution 2,00,000 less share of loss 13,719 (Notes 3A + 3B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Balance Sheet - Other Provisions - Others</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>450000</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Provisions as per Tally (Note 7A)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>B. Corrections to make in Winman (ITR-5, A.Y. 2026-27)</t>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Balance Sheet - Other current assets (sub-table): Receivable from partners</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Capital contribution receivable (Note 10A)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>Winman sheet / field</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>As exported</t>
-        </is>
-      </c>
-      <c r="C19" s="20" t="inlineStr">
-        <is>
-          <t>Change to</t>
-        </is>
-      </c>
-      <c r="D19" s="17" t="inlineStr">
-        <is>
-          <t>Reason</t>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Balance Sheet - Loans &amp; advances - Advances</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>409311</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>409312</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Tally 4,09,311.61 rounded to the nearest rupee</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Balance Sheet - Partners' / Members' capital</t>
+          <t>Balance Sheet - Loans &amp; advances - Balance with Revenue Authorities</t>
         </is>
       </c>
       <c r="B20" s="21" t="inlineStr">
@@ -1954,188 +1979,110 @@
         </is>
       </c>
       <c r="C20" s="21" t="n">
-        <v>186281</v>
+        <v>18475</v>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Contribution 2,00,000 less share of loss 13,719 (Notes 3A + 3B)</t>
+          <t>TDS 2025-26 receivable (Tally)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Balance Sheet - Unsecured loans - Others</t>
-        </is>
-      </c>
-      <c r="B21" s="21" t="inlineStr">
-        <is>
-          <t>(blank)</t>
-        </is>
+          <t>Balance Sheet - Cash / cash equivalents - Balances with Banks</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>45672</v>
       </c>
       <c r="C21" s="21" t="n">
-        <v>250000</v>
+        <v>45673</v>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Long-term interest-free loan from Samartha (Note 5)</t>
+          <t>Tally 45,672.76 rounded to the nearest rupee</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Balance Sheet - Additional data - Unsecured Rupee Loans from persons u/s 40A(2)(b)</t>
-        </is>
-      </c>
-      <c r="B22" s="21" t="inlineStr">
-        <is>
-          <t>(blank)</t>
-        </is>
+          <t>Balance Sheet - Cash / cash equivalents - Others</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>18475</v>
       </c>
       <c r="C22" s="21" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Samartha is a partner - a specified person u/s 40A(2)(b)</t>
+          <t>This is TDS receivable, not cash</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Balance Sheet - Loans &amp; advances - Advances</t>
+          <t>Balance Sheet - Profit and loss A/c (Dr)</t>
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>409311</v>
+        <v>13721</v>
       </c>
       <c r="C23" s="21" t="n">
-        <v>409312</v>
+        <v>0</v>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Tally 4,09,311.61 rounded to the nearest rupee</t>
+          <t>Loss transferred to partners' current accounts (included in capital above)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Balance Sheet - Loans &amp; advances - Balance with Revenue Authorities</t>
-        </is>
-      </c>
-      <c r="B24" s="21" t="inlineStr">
-        <is>
-          <t>(blank)</t>
-        </is>
+          <t>P&amp;L - Sale of products/goods</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>923729</v>
       </c>
       <c r="C24" s="21" t="n">
-        <v>18475</v>
+        <v>0</v>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>TDS 2025-26 receivable (Tally)</t>
+          <t>Sponsorship income is a service</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Balance Sheet - Cash / cash equivalents - Balances with Banks</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>45672</v>
+          <t>P&amp;L - Sale of services (excluding Professional receipts)</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
       </c>
       <c r="C25" s="21" t="n">
-        <v>45673</v>
+        <v>923729</v>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Tally 45,672.76 rounded to the nearest rupee</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Balance Sheet - Cash / cash equivalents - Others</t>
-        </is>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>18475</v>
-      </c>
-      <c r="C26" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>This is TDS receivable, not cash</t>
+          <t>Sponsorship Amount (Tally)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Balance Sheet - Profit and loss A/c (Dr)</t>
-        </is>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>13721</v>
-      </c>
-      <c r="C27" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Loss transferred to partners' current accounts (included in capital above)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>P&amp;L - Sale of products/goods</t>
-        </is>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>923729</v>
-      </c>
-      <c r="C28" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Sponsorship income is a service</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>P&amp;L - Sale of services (excluding Professional receipts)</t>
-        </is>
-      </c>
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>(blank)</t>
-        </is>
-      </c>
-      <c r="C29" s="21" t="n">
-        <v>923729</v>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Sponsorship Amount (Tally)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Everything else in Winman (expenses 9,37,448, trade creditors 28,229, other payables 8,950) already matches and needs no change. After these corrections Winman's Balance Sheet totals 4,73,460 on both sides.</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Everything else in Winman (expenses 9,37,448, trade creditors 28,229, other payables 8,950) already matches and needs no change. After these corrections Winman's Balance Sheet totals 6,73,460 on both sides.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FY 2025-26 financials: show Tally ledger names for provisions
Note 7A now lists Branding Charges Payable and Business Promotion
Payable (Rs 2,25,000 each) as in the detailed Tally trial balance; the
reconciliation names the two trade creditors. No figures change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PBFJrzW3fVaXJi95GNnthu
</commit_message>
<xml_diff>
--- a/outputs/Star_Fandom_FY2025-26_Tally_vs_Financials_vs_Winman.xlsx
+++ b/outputs/Star_Fandom_FY2025-26_Tally_vs_Financials_vs_Winman.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Tally TB as exported (TrialBal.xlsx, latest)</t>
+          <t>Tally TB as exported (Trial_balance_as_per_their_tally.xlsx)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -696,7 +696,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Provisions (Tally group) - Short-term provisions</t>
+          <t>Provisions (Tally group): Branding Charges Payable 2,25,000 + Business Promotion Payable 2,25,000</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -730,7 +730,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Sundry creditors / Trade payables</t>
+          <t>Sundry creditors / Trade payables: Bharathi Air Tel 4,623.82 + Cashfree Payments India Pvt Ltd 23,605.51</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -1599,40 +1599,33 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Provisions (Tally group) - Short-term provisions: Tally: credit side of Branding Expense and Business Promotion (2,25,000 each)</t>
+          <t>Receivable from partners (capital contribution): B/f from FY 2024-25; still receivable. Winman: enter under 'Other current assets'</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Receivable from partners (capital contribution): B/f from FY 2024-25; still receivable. Winman: enter under 'Other current assets'</t>
+          <t>Sponsorship Amount - Sale of services: Winman: move 9,23,729 from 'Sale of products/goods' to 'Sale of services'</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>Sponsorship Amount - Sale of services: Winman: move 9,23,729 from 'Sale of products/goods' to 'Sale of services'</t>
+          <t>Mobile Expenses (Telephone): Financials: 3,918.50 less Tally round off 0.22 = 3,918.28, shown as 3,918</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>Mobile Expenses (Telephone): Financials: 3,918.50 less Tally round off 0.22 = 3,918.28, shown as 3,918</t>
+          <t>Column B (Tally as exported) shows a difference of (13,719.42) on the check row only because the loss still sits in Tally's P&amp;L; it moves to the partners' current accounts when entry 2 on sheet 2 is posted.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
-        <is>
-          <t>Column B (Tally as exported) shows a difference of (13,719.42) on the check row only because the loss still sits in Tally's P&amp;L; it moves to the partners' current accounts when entry 2 on sheet 2 is posted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Tally 'after entries' keeps paise; the financials and Winman are in whole rupees (nearest rupee). Winman as exported cut off the paise on Advances (.61) and Bank (.76) - that is the source of the earlier Rs 2 difference.</t>
         </is>

</xml_diff>